<commit_message>
feat: prepare ExcelAlchemy 3.0 API cleanup
</commit_message>
<xml_diff>
--- a/files/portfolio-import-result-en.xlsx
+++ b/files/portfolio-import-result-en.xlsx
@@ -523,7 +523,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
-    <col width="100.1" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="16.9" customWidth="1" min="3" max="3"/>
     <col width="9.1" customWidth="1" min="4" max="4"/>
     <col width="20.8" customWidth="1" min="5" max="5"/>
@@ -616,10 +616,10 @@
       <c r="B4" s="5" t="inlineStr">
         <is>
           <t>1、【Age】Enter a number between 18 and 65.
-2、【Work email】Enter a valid email address
+2、【Work email】Enter a valid email address, such as name@example.com
 3、【Start date】Enter a date in yyyy/mm/dd format
 4、【Status】Enter "Yes" or "No"
-5、【Team】Option not found; check the field comment for valid values
+5、【Team】Select one of the configured options. Valid values include: Engineering，Operations，Sales
 6、【Salary band】The minimum value cannot be greater than the maximum value</t>
         </is>
       </c>

</xml_diff>